<commit_message>
censo_ejemplo.xlsx: eliminar M13-M16 (queda con 12 movimientos)
</commit_message>
<xml_diff>
--- a/censo_ejemplo.xlsx
+++ b/censo_ejemplo.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2" showHorizontalScroll="1" showVerticalScroll="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0" showHorizontalScroll="1" showVerticalScroll="1"/>
   </bookViews>
   <sheets>
     <sheet name="DATOS" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>hora_inicio</t>
   </si>
@@ -66,18 +66,6 @@
     <t>M12</t>
   </si>
   <si>
-    <t>M13</t>
-  </si>
-  <si>
-    <t>M14</t>
-  </si>
-  <si>
-    <t>M15</t>
-  </si>
-  <si>
-    <t>M16</t>
-  </si>
-  <si>
     <t>07:30</t>
   </si>
   <si>
@@ -129,19 +117,19 @@
     <t xml:space="preserve">Calle Ppal</t>
   </si>
   <si>
+    <t>Este-Oeste</t>
+  </si>
+  <si>
+    <t>Oeste-Este</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calle Sec</t>
+  </si>
+  <si>
+    <t>Norte-Sur</t>
+  </si>
+  <si>
     <t>Sur-Norte</t>
-  </si>
-  <si>
-    <t>Norte-Sur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calle Sec</t>
-  </si>
-  <si>
-    <t>Este-Oeste</t>
-  </si>
-  <si>
-    <t>Oeste-Este</t>
   </si>
   <si>
     <t>clave</t>
@@ -209,8 +197,11 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="0" pivotButton="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -782,28 +773,16 @@
       <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" t="s">
-        <v>18</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -841,28 +820,16 @@
       <c r="O2">
         <v>0</v>
       </c>
-      <c r="P2">
-        <v>9</v>
-      </c>
-      <c r="Q2">
-        <v>0</v>
-      </c>
-      <c r="R2">
-        <v>0</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -898,30 +865,18 @@
         <v>0</v>
       </c>
       <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3">
-        <v>0</v>
-      </c>
-      <c r="R3">
-        <v>0</v>
-      </c>
-      <c r="S3">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
         <v>19</v>
-      </c>
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -959,28 +914,16 @@
       <c r="O4">
         <v>0</v>
       </c>
-      <c r="P4">
-        <v>0</v>
-      </c>
-      <c r="Q4">
-        <v>0</v>
-      </c>
-      <c r="R4">
-        <v>1</v>
-      </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
         <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>24</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -1018,28 +961,16 @@
       <c r="O5">
         <v>0</v>
       </c>
-      <c r="P5">
-        <v>0</v>
-      </c>
-      <c r="Q5">
-        <v>0</v>
-      </c>
-      <c r="R5">
-        <v>0</v>
-      </c>
-      <c r="S5">
-        <v>0</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1077,28 +1008,16 @@
       <c r="O6">
         <v>0</v>
       </c>
-      <c r="P6">
-        <v>8</v>
-      </c>
-      <c r="Q6">
-        <v>0</v>
-      </c>
-      <c r="R6">
-        <v>1</v>
-      </c>
-      <c r="S6">
-        <v>0</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -1134,30 +1053,18 @@
         <v>0</v>
       </c>
       <c r="O7">
-        <v>0</v>
-      </c>
-      <c r="P7">
-        <v>0</v>
-      </c>
-      <c r="Q7">
-        <v>0</v>
-      </c>
-      <c r="R7">
-        <v>0</v>
-      </c>
-      <c r="S7">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -1195,28 +1102,16 @@
       <c r="O8">
         <v>0</v>
       </c>
-      <c r="P8">
-        <v>0</v>
-      </c>
-      <c r="Q8">
-        <v>1</v>
-      </c>
-      <c r="R8">
-        <v>0</v>
-      </c>
-      <c r="S8">
-        <v>0</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
         <v>20</v>
-      </c>
-      <c r="B9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" t="s">
-        <v>24</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -1254,28 +1149,16 @@
       <c r="O9">
         <v>0</v>
       </c>
-      <c r="P9">
-        <v>0</v>
-      </c>
-      <c r="Q9">
-        <v>0</v>
-      </c>
-      <c r="R9">
-        <v>0</v>
-      </c>
-      <c r="S9">
-        <v>0</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -1313,28 +1196,16 @@
       <c r="O10">
         <v>0</v>
       </c>
-      <c r="P10">
-        <v>7</v>
-      </c>
-      <c r="Q10">
-        <v>1</v>
-      </c>
-      <c r="R10">
-        <v>0</v>
-      </c>
-      <c r="S10">
-        <v>0</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -1370,30 +1241,18 @@
         <v>0</v>
       </c>
       <c r="O11">
-        <v>0</v>
-      </c>
-      <c r="P11">
-        <v>0</v>
-      </c>
-      <c r="Q11">
-        <v>0</v>
-      </c>
-      <c r="R11">
-        <v>0</v>
-      </c>
-      <c r="S11">
         <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -1431,28 +1290,16 @@
       <c r="O12">
         <v>0</v>
       </c>
-      <c r="P12">
-        <v>0</v>
-      </c>
-      <c r="Q12">
-        <v>0</v>
-      </c>
-      <c r="R12">
-        <v>0</v>
-      </c>
-      <c r="S12">
-        <v>0</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -1490,28 +1337,16 @@
       <c r="O13">
         <v>0</v>
       </c>
-      <c r="P13">
-        <v>0</v>
-      </c>
-      <c r="Q13">
-        <v>0</v>
-      </c>
-      <c r="R13">
-        <v>0</v>
-      </c>
-      <c r="S13">
-        <v>0</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -1549,28 +1384,16 @@
       <c r="O14">
         <v>0</v>
       </c>
-      <c r="P14">
-        <v>3</v>
-      </c>
-      <c r="Q14">
-        <v>0</v>
-      </c>
-      <c r="R14">
-        <v>0</v>
-      </c>
-      <c r="S14">
-        <v>0</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -1606,30 +1429,18 @@
         <v>0</v>
       </c>
       <c r="O15">
-        <v>0</v>
-      </c>
-      <c r="P15">
-        <v>0</v>
-      </c>
-      <c r="Q15">
-        <v>0</v>
-      </c>
-      <c r="R15">
-        <v>0</v>
-      </c>
-      <c r="S15">
         <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C16" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D16">
         <v>0</v>
@@ -1667,28 +1478,16 @@
       <c r="O16">
         <v>0</v>
       </c>
-      <c r="P16">
-        <v>0</v>
-      </c>
-      <c r="Q16">
-        <v>0</v>
-      </c>
-      <c r="R16">
-        <v>0</v>
-      </c>
-      <c r="S16">
-        <v>0</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D17">
         <v>0</v>
@@ -1726,28 +1525,16 @@
       <c r="O17">
         <v>0</v>
       </c>
-      <c r="P17">
-        <v>0</v>
-      </c>
-      <c r="Q17">
-        <v>0</v>
-      </c>
-      <c r="R17">
-        <v>0</v>
-      </c>
-      <c r="S17">
-        <v>0</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -1785,28 +1572,16 @@
       <c r="O18">
         <v>0</v>
       </c>
-      <c r="P18">
-        <v>7</v>
-      </c>
-      <c r="Q18">
-        <v>0</v>
-      </c>
-      <c r="R18">
-        <v>0</v>
-      </c>
-      <c r="S18">
-        <v>0</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D19">
         <v>0</v>
@@ -1842,30 +1617,18 @@
         <v>0</v>
       </c>
       <c r="O19">
-        <v>0</v>
-      </c>
-      <c r="P19">
-        <v>0</v>
-      </c>
-      <c r="Q19">
-        <v>0</v>
-      </c>
-      <c r="R19">
-        <v>0</v>
-      </c>
-      <c r="S19">
         <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -1903,28 +1666,16 @@
       <c r="O20">
         <v>0</v>
       </c>
-      <c r="P20">
-        <v>0</v>
-      </c>
-      <c r="Q20">
-        <v>0</v>
-      </c>
-      <c r="R20">
-        <v>0</v>
-      </c>
-      <c r="S20">
-        <v>0</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D21">
         <v>0</v>
@@ -1962,28 +1713,16 @@
       <c r="O21">
         <v>0</v>
       </c>
-      <c r="P21">
-        <v>0</v>
-      </c>
-      <c r="Q21">
-        <v>0</v>
-      </c>
-      <c r="R21">
-        <v>0</v>
-      </c>
-      <c r="S21">
-        <v>0</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C22" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -2021,28 +1760,16 @@
       <c r="O22">
         <v>0</v>
       </c>
-      <c r="P22">
-        <v>4</v>
-      </c>
-      <c r="Q22">
-        <v>0</v>
-      </c>
-      <c r="R22">
-        <v>2</v>
-      </c>
-      <c r="S22">
-        <v>0</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C23" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -2078,30 +1805,18 @@
         <v>0</v>
       </c>
       <c r="O23">
-        <v>0</v>
-      </c>
-      <c r="P23">
-        <v>0</v>
-      </c>
-      <c r="Q23">
-        <v>0</v>
-      </c>
-      <c r="R23">
-        <v>0</v>
-      </c>
-      <c r="S23">
         <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C24" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D24">
         <v>0</v>
@@ -2139,28 +1854,16 @@
       <c r="O24">
         <v>0</v>
       </c>
-      <c r="P24">
-        <v>0</v>
-      </c>
-      <c r="Q24">
-        <v>0</v>
-      </c>
-      <c r="R24">
-        <v>0</v>
-      </c>
-      <c r="S24">
-        <v>0</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -2198,28 +1901,16 @@
       <c r="O25">
         <v>0</v>
       </c>
-      <c r="P25">
-        <v>0</v>
-      </c>
-      <c r="Q25">
-        <v>0</v>
-      </c>
-      <c r="R25">
-        <v>0</v>
-      </c>
-      <c r="S25">
-        <v>0</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C26" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D26">
         <v>0</v>
@@ -2257,28 +1948,16 @@
       <c r="O26">
         <v>0</v>
       </c>
-      <c r="P26">
-        <v>3</v>
-      </c>
-      <c r="Q26">
-        <v>0</v>
-      </c>
-      <c r="R26">
-        <v>0</v>
-      </c>
-      <c r="S26">
-        <v>0</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C27" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -2314,30 +1993,18 @@
         <v>0</v>
       </c>
       <c r="O27">
-        <v>0</v>
-      </c>
-      <c r="P27">
-        <v>0</v>
-      </c>
-      <c r="Q27">
-        <v>0</v>
-      </c>
-      <c r="R27">
-        <v>0</v>
-      </c>
-      <c r="S27">
         <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C28" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D28">
         <v>0</v>
@@ -2375,28 +2042,16 @@
       <c r="O28">
         <v>0</v>
       </c>
-      <c r="P28">
-        <v>2</v>
-      </c>
-      <c r="Q28">
-        <v>0</v>
-      </c>
-      <c r="R28">
-        <v>0</v>
-      </c>
-      <c r="S28">
-        <v>0</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B29" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C29" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D29">
         <v>0</v>
@@ -2434,28 +2089,16 @@
       <c r="O29">
         <v>0</v>
       </c>
-      <c r="P29">
-        <v>0</v>
-      </c>
-      <c r="Q29">
-        <v>0</v>
-      </c>
-      <c r="R29">
-        <v>0</v>
-      </c>
-      <c r="S29">
-        <v>0</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B30" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C30" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -2493,28 +2136,16 @@
       <c r="O30">
         <v>0</v>
       </c>
-      <c r="P30">
-        <v>2</v>
-      </c>
-      <c r="Q30">
-        <v>0</v>
-      </c>
-      <c r="R30">
-        <v>1</v>
-      </c>
-      <c r="S30">
-        <v>0</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C31" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -2550,30 +2181,18 @@
         <v>0</v>
       </c>
       <c r="O31">
-        <v>0</v>
-      </c>
-      <c r="P31">
-        <v>0</v>
-      </c>
-      <c r="Q31">
-        <v>0</v>
-      </c>
-      <c r="R31">
-        <v>0</v>
-      </c>
-      <c r="S31">
         <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B32" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C32" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -2611,28 +2230,16 @@
       <c r="O32">
         <v>0</v>
       </c>
-      <c r="P32">
-        <v>0</v>
-      </c>
-      <c r="Q32">
-        <v>0</v>
-      </c>
-      <c r="R32">
-        <v>0</v>
-      </c>
-      <c r="S32">
-        <v>0</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C33" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D33">
         <v>0</v>
@@ -2668,18 +2275,6 @@
         <v>0</v>
       </c>
       <c r="O33">
-        <v>0</v>
-      </c>
-      <c r="P33">
-        <v>0</v>
-      </c>
-      <c r="Q33">
-        <v>0</v>
-      </c>
-      <c r="R33">
-        <v>0</v>
-      </c>
-      <c r="S33">
         <v>0</v>
       </c>
     </row>
@@ -2697,17 +2292,20 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="3" width="24.8515625"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2">
@@ -2715,10 +2313,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -2726,10 +2324,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
@@ -2737,10 +2335,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
@@ -2748,10 +2346,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6">
@@ -2759,10 +2357,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -2770,10 +2368,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8">
@@ -2781,10 +2379,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
         <v>35</v>
-      </c>
-      <c r="C8" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="9">
@@ -2792,10 +2390,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
         <v>35</v>
-      </c>
-      <c r="C9" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="10">
@@ -2803,10 +2401,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" t="s">
-        <v>39</v>
+        <v>34</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="11">
@@ -2814,10 +2412,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12">
@@ -2825,10 +2423,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13">
@@ -2836,54 +2434,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" t="s">
-        <v>38</v>
-      </c>
-      <c r="C16" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -2907,50 +2461,50 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>